<commit_message>
Add missing functionality and excel tests.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_interpolatedyieldcurves.xlsx
+++ b/tests/workbooktests/workbooks/test_interpolatedyieldcurves.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8DF0BA-D446-44AA-B300-0D74EA0F58AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CF52CE-ABF6-4D4A-8C88-776FDE91B73E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{5088EC6F-18E0-4AC9-9BC5-4CE1169B8F7F}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="30930" windowHeight="16770" xr2:uid="{5088EC6F-18E0-4AC9-9BC5-4CE1169B8F7F}"/>
   </bookViews>
   <sheets>
     <sheet name="qlInterpolatedYieldCurve" sheetId="1" r:id="rId1"/>
@@ -20,44 +20,11 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -136,7 +103,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,7 +138,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -504,14 +471,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38FE1B30-2282-4CB0-BC3A-F4A304EAB6FC}">
   <dimension ref="A2:D40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="21.5546875" customWidth="1"/>
-    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
+    <col min="2" max="2" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -519,7 +486,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -530,10 +497,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4">
       <c r="B5" s="1">
         <f ca="1">TODAY()</f>
-        <v>46245</v>
+        <v>46279</v>
       </c>
       <c r="C5" s="2">
         <f ca="1">EXP(-$C$2*(B5-$B$5)/365)</f>
@@ -544,63 +511,63 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4">
       <c r="B6" s="1">
         <f ca="1">B5+365</f>
-        <v>46610</v>
+        <v>46644</v>
       </c>
       <c r="C6" s="2">
         <f ca="1">EXP(-$C$2*(B6-$B$5)/365)</f>
         <v>0.97044553354850815</v>
       </c>
       <c r="D6">
-        <f t="shared" ref="D6:D9" si="0">$C$2</f>
+        <f>$C$2</f>
         <v>0.03</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4">
       <c r="B7" s="1">
         <f ca="1">B6+365</f>
-        <v>46975</v>
+        <v>47009</v>
       </c>
       <c r="C7" s="2">
         <f ca="1">EXP(-$C$2*(B7-$B$5)/365)</f>
         <v>0.94176453358424872</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
+        <f>$C$2</f>
         <v>0.03</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4">
       <c r="B8" s="1">
         <f ca="1">B7+365</f>
-        <v>47340</v>
+        <v>47374</v>
       </c>
       <c r="C8" s="2">
         <f ca="1">EXP(-$C$2*(B8-$B$5)/365)</f>
         <v>0.91393118527122819</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
+        <f>$C$2</f>
         <v>0.03</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4">
       <c r="B9" s="1">
         <f ca="1">B8+365</f>
-        <v>47705</v>
+        <v>47739</v>
       </c>
       <c r="C9" s="2">
         <f ca="1">EXP(-$C$2*(B9-$B$5)/365)</f>
         <v>0.88692043671715748</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
+        <f>$C$2</f>
         <v>0.03</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -608,7 +575,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -616,7 +583,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -624,17 +591,17 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4">
       <c r="C15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4">
       <c r="C16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -642,123 +609,123 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="C19" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="C20" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="C21" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="C22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="C23" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>7</v>
       </c>
-      <c r="C25" t="str" cm="1">
+      <c r="C25" t="str">
         <f t="array" aca="1" ref="C25" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$14,C18)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R25C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C26" t="str" cm="1">
+    <row r="26" spans="1:3">
+      <c r="C26" t="str">
         <f t="array" aca="1" ref="C26" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$14,C19)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R26C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C27" t="str" cm="1">
+    <row r="27" spans="1:3">
+      <c r="C27" t="str">
         <f t="array" aca="1" ref="C27" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$14,C20)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R27C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>7</v>
       </c>
-      <c r="C29" t="str" cm="1">
+      <c r="C29" t="str">
         <f t="array" aca="1" ref="C29" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$15,C18)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R29C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C30" t="str" cm="1">
+    <row r="30" spans="1:3">
+      <c r="C30" t="str">
         <f t="array" aca="1" ref="C30" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$15,C19)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R30C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C31" t="str" cm="1">
+    <row r="31" spans="1:3">
+      <c r="C31" t="str">
         <f t="array" aca="1" ref="C31" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$15,C21)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R31C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C32" t="str" cm="1">
+    <row r="32" spans="1:3">
+      <c r="C32" t="str">
         <f t="array" aca="1" ref="C32" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$15,C22)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R32C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>7</v>
       </c>
-      <c r="C34" t="str" cm="1">
+      <c r="C34" t="str">
         <f t="array" aca="1" ref="C34" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$16,C18)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R34C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C35" t="str" cm="1">
+    <row r="35" spans="1:3">
+      <c r="C35" t="str">
         <f t="array" aca="1" ref="C35" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$16,C19)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R35C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C36" t="str" cm="1">
+    <row r="36" spans="1:3">
+      <c r="C36" t="str">
         <f t="array" aca="1" ref="C36" ca="1">_xll.qlInterpolatedYieldCurve($B$5:$B$9,$C$5:$C$9,$C$11,$C$12,$C$16,C23)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R36C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3">
       <c r="A38" t="s">
         <v>19</v>
       </c>
-      <c r="C38" t="str" cm="1">
-        <f t="array" aca="1" ref="C38" ca="1">_xll.qlDiscountCurve(B5:B9,C5:C9)</f>
-        <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R38C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C38" t="str">
+        <f t="array" aca="1" ref="C38" ca="1">_xll.qlDiscountCurve(B5:B9,C5:C9,"actual365fixed")</f>
+        <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R38C3YieldTermStructureHandle,E</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="A39" t="s">
         <v>20</v>
       </c>
-      <c r="C39" t="str" cm="1">
+      <c r="C39" t="str">
         <f t="array" aca="1" ref="C39" ca="1">_xll.qlForwardCurve(B5:B9,D5:D9,C11)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R39C3YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3">
       <c r="A40" t="s">
         <v>21</v>
       </c>
-      <c r="C40" t="str" cm="1">
+      <c r="C40" t="str">
         <f t="array" aca="1" ref="C40" ca="1">_xll.qlZeroCurve(B5:B9,D5:D9,,C12)</f>
         <v>欣[test_interpolatedyieldcurves.xlsx]qlInterpolatedYieldCurve!R40C3YieldTermStructureHandle,A</v>
       </c>

</xml_diff>